<commit_message>
sn: sppa update forms
</commit_message>
<xml_diff>
--- a/SCH-STH/Impact assessments/Senegal/2025/octobre/sn_sppa_impact_2510_2_child.xlsx
+++ b/SCH-STH/Impact assessments/Senegal/2025/octobre/sn_sppa_impact_2510_2_child.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\SCH-STH\Impact assessments\Senegal\2025\octobre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE4656A-D5FA-4029-ABAD-F6491644CB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FCCFF0-B269-4E8A-993B-6FEB83D9E085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2099,10 +2099,10 @@
       </c>
       <c r="K17" s="66"/>
       <c r="L17" s="66"/>
-      <c r="M17" s="66"/>
-      <c r="N17" s="65" t="s">
+      <c r="M17" s="65" t="s">
         <v>13</v>
       </c>
+      <c r="N17" s="65"/>
       <c r="O17" s="67"/>
     </row>
     <row r="18" spans="1:21" s="28" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">

</xml_diff>